<commit_message>
chore(resources): update mappings template workbook
</commit_message>
<xml_diff>
--- a/resources/mappings_template.xlsx
+++ b/resources/mappings_template.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PedroPauloFavatoBarc\Dev\semantic-interoperability\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F706728F-8092-4787-8AA1-4A630632A84F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF18857B-3203-431C-9144-260A29CAA2C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A1364C1B-3702-4249-8DB4-2D82861A95E3}"/>
+    <workbookView xWindow="28680" yWindow="-1485" windowWidth="29040" windowHeight="16440" xr2:uid="{A1364C1B-3702-4249-8DB4-2D82861A95E3}"/>
   </bookViews>
   <sheets>
     <sheet name="Mappings" sheetId="1" r:id="rId1"/>
     <sheet name="Prefixes" sheetId="2" r:id="rId2"/>
     <sheet name="Hash" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet name="Basic Info" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="89">
   <si>
     <t>subject_id</t>
   </si>
@@ -182,13 +183,216 @@
   </si>
   <si>
     <t>https://w3id.org/sssom/</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/</t>
+  </si>
+  <si>
+    <t>obo</t>
+  </si>
+  <si>
+    <t>care-sm</t>
+  </si>
+  <si>
+    <t>https://w3id.org/CARE-SM#</t>
+  </si>
+  <si>
+    <t>fhir</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/</t>
+  </si>
+  <si>
+    <t>hl7</t>
+  </si>
+  <si>
+    <t>http://terminology.hl7.org/ValueSet/</t>
+  </si>
+  <si>
+    <t>hri-cdash</t>
+  </si>
+  <si>
+    <t>https://data.health-ri.nl/id/cdash/</t>
+  </si>
+  <si>
+    <t>hri-fhir-r5</t>
+  </si>
+  <si>
+    <t>https://data.health-ri.nl/id/fhir-r5/</t>
+  </si>
+  <si>
+    <t>hri-ga4gh-phenopacket-schema</t>
+  </si>
+  <si>
+    <t>https://data.health-ri.nl/id/ga4gh-phenopacket-schema/</t>
+  </si>
+  <si>
+    <t>hri-icd11</t>
+  </si>
+  <si>
+    <t>https://data.health-ri.nl/id/icd11/</t>
+  </si>
+  <si>
+    <t>hri-omop</t>
+  </si>
+  <si>
+    <t>https://data.health-ri.nl/id/omop/</t>
+  </si>
+  <si>
+    <t>hri-openehr</t>
+  </si>
+  <si>
+    <t>https://data.health-ri.nl/id/openehr/</t>
+  </si>
+  <si>
+    <t>loinc</t>
+  </si>
+  <si>
+    <t>https://loinc.org/</t>
+  </si>
+  <si>
+    <t>mesh</t>
+  </si>
+  <si>
+    <t>http://purl.bioontology.org/ontology/MESH/</t>
+  </si>
+  <si>
+    <t>ncit</t>
+  </si>
+  <si>
+    <t>https://evsexplore.semantics.cancer.gov/evsexplore/concept/ncit/</t>
+  </si>
+  <si>
+    <t>snomed</t>
+  </si>
+  <si>
+    <t>http://snomed.info/id/</t>
+  </si>
+  <si>
+    <t>Meaning</t>
+  </si>
+  <si>
+    <t>Background Color</t>
+  </si>
+  <si>
+    <t>TEMPLATE COLORING LEGEND</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>optional</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> are green</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>mandatory</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> with a variable default are purple and not pre-filled</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>mandatory</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> with a fixed default are purple and pre-filled</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>mandatory</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> with no default have a black background</t>
+    </r>
+  </si>
+  <si>
+    <t>Author</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Version</t>
+  </si>
+  <si>
+    <t>2.1.0</t>
+  </si>
+  <si>
+    <t>Pedro Paulo F. Barcelos</t>
+  </si>
+  <si>
+    <t>METADATA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -204,8 +408,24 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -242,8 +462,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -251,12 +489,109 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -265,12 +600,37 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="29">
+  <dxfs count="59">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -283,6 +643,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -293,6 +673,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFEB9C"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF9C5700"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -302,6 +702,59 @@
       </fill>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9F9F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFEB9C"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF9C5700"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <color rgb="FF9C5700"/>
       </font>
@@ -315,6 +768,207 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFF9F9F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFEB9C"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF9C5700"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9F9F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFEB9C"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF9C5700"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9F9F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFEB9C"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF9C5700"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9F9F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9F9F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -328,9 +982,6 @@
           <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <font>
@@ -842,10 +1493,10 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF9C5700"/>
+      <color rgb="FFFFEB9C"/>
       <color rgb="FFFF9F9F"/>
       <color rgb="FFFFE1E1"/>
-      <color rgb="FFFFEB9C"/>
-      <color rgb="FF9C5700"/>
     </mruColors>
   </colors>
   <extLst>
@@ -860,41 +1511,44 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F3A1F876-3ACD-4118-8509-5D77BAD95681}" name="Table1" displayName="Table1" ref="A1:X4" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F3A1F876-3ACD-4118-8509-5D77BAD95681}" name="Table1" displayName="Table1" ref="A1:X4" totalsRowShown="0" headerRowDxfId="58" dataDxfId="57">
   <autoFilter ref="A1:X4" xr:uid="{F3A1F876-3ACD-4118-8509-5D77BAD95681}"/>
   <tableColumns count="24">
-    <tableColumn id="1" xr3:uid="{418DF1C6-46AE-4D05-8CFD-E9533A5BC2B0}" name="record_id" dataDxfId="26"/>
-    <tableColumn id="2" xr3:uid="{5629DEAA-C64A-4C26-9C3D-441AA1987215}" name="subject_id" dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{418DF1C6-46AE-4D05-8CFD-E9533A5BC2B0}" name="record_id" dataDxfId="56"/>
+    <tableColumn id="2" xr3:uid="{5629DEAA-C64A-4C26-9C3D-441AA1987215}" name="subject_id" dataDxfId="55"/>
     <tableColumn id="24" xr3:uid="{E31C51FF-F9AD-475F-9F4C-5928C1897048}" name="subject_label" dataCellStyle="Normal"/>
     <tableColumn id="23" xr3:uid="{CE7AF749-7B4B-4226-8150-13024DD6295F}" name="predicate_id"/>
     <tableColumn id="22" xr3:uid="{D6FFE393-4DC9-49A9-9C9B-0BA6E4351B72}" name="predicate_modifier"/>
-    <tableColumn id="3" xr3:uid="{5DE55A22-49F3-4CE4-92AB-E4082CDB5810}" name="object_id" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{5DE55A22-49F3-4CE4-92AB-E4082CDB5810}" name="object_id" dataDxfId="54"/>
     <tableColumn id="18" xr3:uid="{F897D13D-6D73-46AE-91CB-FF641F299710}" name="object_label" dataCellStyle="Normal"/>
-    <tableColumn id="4" xr3:uid="{0A81517D-DEC8-44BF-8F85-5FF7FE98F200}" name="object_category" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{26DBBA81-542B-4F93-83EE-28068E94BE05}" name="mapping_justification" dataDxfId="22"/>
-    <tableColumn id="6" xr3:uid="{1A470CAB-4A9A-4541-AE74-B2B9A03DD29E}" name="author_id" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{0A81517D-DEC8-44BF-8F85-5FF7FE98F200}" name="object_category" dataDxfId="53"/>
+    <tableColumn id="5" xr3:uid="{26DBBA81-542B-4F93-83EE-28068E94BE05}" name="mapping_justification" dataDxfId="52"/>
+    <tableColumn id="6" xr3:uid="{1A470CAB-4A9A-4541-AE74-B2B9A03DD29E}" name="author_id" dataDxfId="51"/>
     <tableColumn id="25" xr3:uid="{4D5897AE-98CC-421A-8916-FA23AC9E84FD}" name="author_label"/>
-    <tableColumn id="7" xr3:uid="{DF2F500D-9154-4455-B03E-CC2B6739AE84}" name="reviewer_id" dataDxfId="20"/>
-    <tableColumn id="8" xr3:uid="{499DBD21-2B5A-4A38-9FFA-0477EF18EC6A}" name="reviewer_label" dataDxfId="19"/>
-    <tableColumn id="9" xr3:uid="{72FCD242-C99E-40FF-9358-9CCD02E5EDFA}" name="creator_id" dataDxfId="18"/>
-    <tableColumn id="10" xr3:uid="{899C370E-BA5B-4C4B-927A-CFBD3F409FDE}" name="creator_label" dataDxfId="17"/>
-    <tableColumn id="11" xr3:uid="{F6634A69-4617-4282-808A-1A99C1B24438}" name="license" dataDxfId="16"/>
-    <tableColumn id="12" xr3:uid="{3D7D04A3-334E-46BD-A964-B3690AA2C5D6}" name="subject_type" dataDxfId="15"/>
-    <tableColumn id="17" xr3:uid="{CBE26A85-1268-4A70-B764-04D3EDB43906}" name="subject_source" dataDxfId="14"/>
-    <tableColumn id="19" xr3:uid="{70B1F6AC-3F94-482D-8586-7E477F4E47BE}" name="subject_source_version" dataDxfId="13"/>
-    <tableColumn id="21" xr3:uid="{D429941D-58EA-4400-8BD7-CF5541B8B709}" name="object_source_version" dataDxfId="12"/>
-    <tableColumn id="26" xr3:uid="{8683B23B-85C0-4581-9D45-264D7BAE8FEE}" name="mapping_date" dataDxfId="11"/>
-    <tableColumn id="27" xr3:uid="{92D3255A-1ACB-4AE8-A5F9-358B77734284}" name="publication_date" dataDxfId="10"/>
-    <tableColumn id="28" xr3:uid="{5154C138-4F05-4AD2-81D2-9BB957CAFC21}" name="comment" dataDxfId="9"/>
-    <tableColumn id="29" xr3:uid="{8922DC1B-E4F4-4E06-9EF7-B4ADE68C21FE}" name="replaces" dataDxfId="8"/>
+    <tableColumn id="7" xr3:uid="{DF2F500D-9154-4455-B03E-CC2B6739AE84}" name="reviewer_id" dataDxfId="50"/>
+    <tableColumn id="8" xr3:uid="{499DBD21-2B5A-4A38-9FFA-0477EF18EC6A}" name="reviewer_label" dataDxfId="49"/>
+    <tableColumn id="9" xr3:uid="{72FCD242-C99E-40FF-9358-9CCD02E5EDFA}" name="creator_id" dataDxfId="48"/>
+    <tableColumn id="10" xr3:uid="{899C370E-BA5B-4C4B-927A-CFBD3F409FDE}" name="creator_label" dataDxfId="47"/>
+    <tableColumn id="11" xr3:uid="{F6634A69-4617-4282-808A-1A99C1B24438}" name="license" dataDxfId="46"/>
+    <tableColumn id="12" xr3:uid="{3D7D04A3-334E-46BD-A964-B3690AA2C5D6}" name="subject_type" dataDxfId="45"/>
+    <tableColumn id="17" xr3:uid="{CBE26A85-1268-4A70-B764-04D3EDB43906}" name="subject_source" dataDxfId="44"/>
+    <tableColumn id="19" xr3:uid="{70B1F6AC-3F94-482D-8586-7E477F4E47BE}" name="subject_source_version" dataDxfId="43"/>
+    <tableColumn id="21" xr3:uid="{D429941D-58EA-4400-8BD7-CF5541B8B709}" name="object_source_version" dataDxfId="42"/>
+    <tableColumn id="26" xr3:uid="{8683B23B-85C0-4581-9D45-264D7BAE8FEE}" name="mapping_date" dataDxfId="41"/>
+    <tableColumn id="27" xr3:uid="{92D3255A-1ACB-4AE8-A5F9-358B77734284}" name="publication_date" dataDxfId="40"/>
+    <tableColumn id="28" xr3:uid="{5154C138-4F05-4AD2-81D2-9BB957CAFC21}" name="comment" dataDxfId="39"/>
+    <tableColumn id="29" xr3:uid="{8922DC1B-E4F4-4E06-9EF7-B4ADE68C21FE}" name="replaces" dataDxfId="38"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium18" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{CB1467CD-C73D-4100-B5C5-5FDBC07F3BC9}" name="Table2" displayName="Table2" ref="A1:B9" totalsRowShown="0">
-  <autoFilter ref="A1:B9" xr:uid="{CB1467CD-C73D-4100-B5C5-5FDBC07F3BC9}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{CB1467CD-C73D-4100-B5C5-5FDBC07F3BC9}" name="Table2" displayName="Table2" ref="A1:B23" totalsRowShown="0">
+  <autoFilter ref="A1:B23" xr:uid="{CB1467CD-C73D-4100-B5C5-5FDBC07F3BC9}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B10">
+    <sortCondition ref="A1:A10"/>
+  </sortState>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{BC5BD901-C15C-4659-ACC7-AE3A02A88257}" name="Prefix"/>
     <tableColumn id="2" xr3:uid="{9FD0CC88-7BCF-44DD-917A-4DCFF0710D03}" name="URI"/>
@@ -904,51 +1558,29 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{20FEFA3C-87BD-4761-9EAB-32AE51ADFEC7}" name="Table3" displayName="Table3" ref="A1:X4" totalsRowShown="0">
-  <autoFilter ref="A1:X4" xr:uid="{20FEFA3C-87BD-4761-9EAB-32AE51ADFEC7}"/>
-  <tableColumns count="24">
-    <tableColumn id="1" xr3:uid="{4FDD882A-7228-421A-AA68-F64B4A19C43C}" name="record_id"/>
-    <tableColumn id="2" xr3:uid="{D0AF222F-2301-4B65-8CB4-7706D2873BC0}" name="subject_id"/>
-    <tableColumn id="3" xr3:uid="{D335C766-4703-4450-82BC-371143873D2C}" name="subject_label"/>
-    <tableColumn id="4" xr3:uid="{8DDC1DA9-877C-4868-AF20-25CFB369E074}" name="predicate_id"/>
-    <tableColumn id="5" xr3:uid="{C9D0BF3C-E311-4533-9A0D-BF02475CC0DF}" name="predicate_modifier"/>
-    <tableColumn id="6" xr3:uid="{736DB1AD-7AF7-46CA-A82C-D6B36E8B309A}" name="object_id"/>
-    <tableColumn id="7" xr3:uid="{8E95B2F2-79B4-4DF7-84E3-C9A3B95DAF05}" name="object_label"/>
-    <tableColumn id="8" xr3:uid="{4F13B562-5A39-4A58-ACCD-024F9F21A2BE}" name="object_category"/>
-    <tableColumn id="9" xr3:uid="{F263EFF9-54C4-43DF-B814-398CEFDA72D4}" name="mapping_justification"/>
-    <tableColumn id="10" xr3:uid="{E1F915B8-8E9D-4F6E-AF3D-53E5238EE408}" name="author_id"/>
-    <tableColumn id="11" xr3:uid="{001B78BB-DE8D-41BE-BCC4-D934297A6CEC}" name="author_label"/>
-    <tableColumn id="12" xr3:uid="{6D4EAC80-1AD8-4056-B80C-C5EE7D842D08}" name="reviewer_id"/>
-    <tableColumn id="13" xr3:uid="{7428200C-BD5D-4596-99BC-13F516330D58}" name="reviewer_label"/>
-    <tableColumn id="14" xr3:uid="{7A3A1692-9BD0-4019-AE48-817739D25975}" name="creator_id"/>
-    <tableColumn id="15" xr3:uid="{F346F4A4-2913-4494-9BBC-38739A8033F5}" name="creator_label"/>
-    <tableColumn id="16" xr3:uid="{9527D45B-717F-4888-9B86-A55EFAADDEDB}" name="license"/>
-    <tableColumn id="17" xr3:uid="{D4B4B6DB-1EEF-4C0E-AFB8-A0CA0BD3DB99}" name="subject_type"/>
-    <tableColumn id="18" xr3:uid="{1372EBD2-4399-4621-90B1-3130F25B9371}" name="subject_source"/>
-    <tableColumn id="19" xr3:uid="{7266452A-F272-43F4-BA27-03EF40AEA97B}" name="subject_source_version"/>
-    <tableColumn id="21" xr3:uid="{BC303C80-F7DB-47AA-AA8B-4EFAB06C137E}" name="object_source_version"/>
-    <tableColumn id="22" xr3:uid="{495885EF-F462-4CEB-BE9F-5E8694B5F395}" name="mapping_date"/>
-    <tableColumn id="23" xr3:uid="{93DC2089-463F-4BB1-B95C-5108C64D5D3B}" name="publication_date"/>
-    <tableColumn id="24" xr3:uid="{520812E4-78A0-4E07-BD50-3994D98373BA}" name="comment"/>
-    <tableColumn id="25" xr3:uid="{DF632399-E8ED-4E1E-AB38-879DE81879EF}" name="replaces"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{DC187EFA-DC60-4013-96D7-B4A7452B0918}" name="Table4" displayName="Table4" ref="A1:C4" totalsRowShown="0">
+  <autoFilter ref="A1:C4" xr:uid="{DC187EFA-DC60-4013-96D7-B4A7452B0918}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{5C1F10EC-45AF-4A89-B63A-8325F9C5D0CE}" name="HASH" dataDxfId="34">
+      <calculatedColumnFormula>_xlfn.CONCAT(Table1[[#This Row],[subject_id]],Table1[[#This Row],[predicate_id]],Table1[[#This Row],[object_id]],Table1[[#This Row],[mapping_justification]],Table1[[#This Row],[author_id]],Table1[[#This Row],[reviewer_id]],Table1[[#This Row],[creator_id]],Table1[[#This Row],[creator_label]],Table1[[#This Row],[license]],Table1[[#This Row],[object_source_version]],Table1[[#This Row],[mapping_date]])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{40455983-5BAF-4A79-A2C8-800C9F6F5778}" name="CRC-32" dataDxfId="37"/>
+    <tableColumn id="2" xr3:uid="{DDBD3CA0-1C5A-4027-AA34-B67FEEF353D2}" name="record_id" dataDxfId="36">
+      <calculatedColumnFormula>"hrim:"&amp;Table4[[#This Row],[CRC-32]]</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium20" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{DC187EFA-DC60-4013-96D7-B4A7452B0918}" name="Table4" displayName="Table4" ref="Z1:AB4" totalsRowShown="0">
-  <autoFilter ref="Z1:AB4" xr:uid="{DC187EFA-DC60-4013-96D7-B4A7452B0918}"/>
-  <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{5C1F10EC-45AF-4A89-B63A-8325F9C5D0CE}" name="HASH" dataDxfId="7">
-      <calculatedColumnFormula>_xlfn.CONCAT(Table3[[#This Row],[mapping_date]])</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="3" xr3:uid="{40455983-5BAF-4A79-A2C8-800C9F6F5778}" name="CRC-32" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{DDBD3CA0-1C5A-4027-AA34-B67FEEF353D2}" name="record_id" dataDxfId="5">
-      <calculatedColumnFormula>"hrim:"&amp;Table4[[#This Row],[CRC-32]]</calculatedColumnFormula>
-    </tableColumn>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{26BC643F-CD39-4B3F-BD65-8AD6D68B0A9C}" name="Table3" displayName="Table3" ref="B8:C12" totalsRowShown="0" tableBorderDxfId="8">
+  <autoFilter ref="B8:C12" xr:uid="{26BC643F-CD39-4B3F-BD65-8AD6D68B0A9C}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{0A32C377-0405-4F3C-A700-6B062BFC484D}" name="Background Color"/>
+    <tableColumn id="2" xr3:uid="{320953A2-F371-4386-8692-9760378CE758}" name="Meaning"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1406,27 +2038,25 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D2:D4 B2:B4 F2:F4 J2:J4 L2:L4">
-    <cfRule type="containsBlanks" dxfId="4" priority="7">
+    <cfRule type="containsBlanks" dxfId="7" priority="7">
       <formula>LEN(TRIM(B2))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D4">
-    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="narrower">
-      <formula>NOT(ISERROR(SEARCH("narrower",D2)))</formula>
+  <conditionalFormatting sqref="D1:E1048576">
+    <cfRule type="expression" dxfId="6" priority="2">
+      <formula>ISNUMBER(SEARCH("narrow",$D1))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="5" operator="containsText" text="broader">
-      <formula>NOT(ISERROR(SEARCH("broader",D2)))</formula>
+    <cfRule type="expression" dxfId="5" priority="3">
+      <formula>ISNUMBER(SEARCH("broader",$D1))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="6" operator="containsText" text="exact">
-      <formula>NOT(ISERROR(SEARCH("exact",D2)))</formula>
+    <cfRule type="expression" dxfId="4" priority="5">
+      <formula>ISNUMBER(SEARCH("not",$E1))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="6">
+      <formula>ISNUMBER(SEARCH("exact",$D1))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E4">
-    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="not">
-      <formula>NOT(ISERROR(SEARCH("not",E2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="20">
+  <dataValidations xWindow="562" yWindow="304" count="20">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid predicate_modifier" error="Leave blank or set to Not (case-sensitive). No other values allowed." promptTitle="About predicate_modifier" prompt="Optional. Leave blank or set to Not to negate the predicate." sqref="E2:E4" xr:uid="{E9C6CA8F-7B41-4974-A5B0-AF180B53928D}">
       <formula1>"Not"</formula1>
     </dataValidation>
@@ -1487,7 +2117,7 @@
   <sheetPr>
     <tabColor theme="5"/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.42578125" customWidth="1"/>
@@ -1504,71 +2134,189 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="B6" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="B7" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="B8" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>62</v>
+      </c>
+      <c r="B9" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>66</v>
+      </c>
+      <c r="B13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>68</v>
+      </c>
+      <c r="B15" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>70</v>
+      </c>
+      <c r="B16" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>72</v>
+      </c>
+      <c r="B17" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>49</v>
+      </c>
+      <c r="B18" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>40</v>
+      </c>
+      <c r="B19" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>74</v>
+      </c>
+      <c r="B22" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>46</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B23" t="s">
         <v>47</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A1:A1048576">
+    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B1:B1048576">
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+  </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B9" xr:uid="{379FEBE4-82E4-4B17-8CE7-0993F7A22FA6}">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B23" xr:uid="{379FEBE4-82E4-4B17-8CE7-0993F7A22FA6}">
       <formula1>AND(ISNUMBER(FIND(":", B2)), FIND(":", B2) &gt; 1, FIND(":", B2) &lt; LEN(B2))</formula1>
     </dataValidation>
   </dataValidations>
@@ -1585,135 +2333,160 @@
   <sheetPr>
     <tabColor rgb="FFC00000"/>
   </sheetPr>
-  <dimension ref="A1:AB4"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="24" width="10.7109375" customWidth="1"/>
-    <col min="26" max="28" width="15.7109375" customWidth="1"/>
+    <col min="1" max="3" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" t="s">
-        <v>20</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H1" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K1" t="s">
-        <v>8</v>
-      </c>
-      <c r="L1" t="s">
-        <v>9</v>
-      </c>
-      <c r="M1" t="s">
-        <v>10</v>
-      </c>
-      <c r="N1" t="s">
-        <v>22</v>
-      </c>
-      <c r="O1" t="s">
-        <v>23</v>
-      </c>
-      <c r="P1" t="s">
-        <v>11</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>12</v>
-      </c>
-      <c r="R1" t="s">
-        <v>13</v>
-      </c>
-      <c r="S1" t="s">
-        <v>14</v>
-      </c>
-      <c r="T1" t="s">
-        <v>24</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="V1" t="s">
-        <v>25</v>
-      </c>
-      <c r="W1" t="s">
-        <v>16</v>
-      </c>
-      <c r="X1" t="s">
-        <v>19</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA1" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="Z2" t="str">
-        <f>_xlfn.CONCAT(Table3[[#This Row],[mapping_date]])</f>
-        <v/>
-      </c>
-      <c r="AA2" s="6"/>
-      <c r="AB2" t="str">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="str">
+        <f>_xlfn.CONCAT(Table1[[#This Row],[subject_id]],Table1[[#This Row],[predicate_id]],Table1[[#This Row],[object_id]],Table1[[#This Row],[mapping_justification]],Table1[[#This Row],[author_id]],Table1[[#This Row],[reviewer_id]],Table1[[#This Row],[creator_id]],Table1[[#This Row],[creator_label]],Table1[[#This Row],[license]],Table1[[#This Row],[object_source_version]],Table1[[#This Row],[mapping_date]])</f>
+        <v>semapv:ManualMappingCurationhttps://w3id.org/health-ri/semantic-interoperabilityHealth-RI Semantic Interoperability Initiativehttps://creativecommons.org/licenses/by/4.0/</v>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" t="str">
         <f>"hrim:"&amp;Table4[[#This Row],[CRC-32]]</f>
         <v>hrim:</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="Z3" t="str">
-        <f>_xlfn.CONCAT(Table3[[#This Row],[mapping_date]])</f>
-        <v/>
-      </c>
-      <c r="AA3" s="6"/>
-      <c r="AB3" t="str">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="str">
+        <f>_xlfn.CONCAT(Table1[[#This Row],[subject_id]],Table1[[#This Row],[predicate_id]],Table1[[#This Row],[object_id]],Table1[[#This Row],[mapping_justification]],Table1[[#This Row],[author_id]],Table1[[#This Row],[reviewer_id]],Table1[[#This Row],[creator_id]],Table1[[#This Row],[creator_label]],Table1[[#This Row],[license]],Table1[[#This Row],[object_source_version]],Table1[[#This Row],[mapping_date]])</f>
+        <v>semapv:ManualMappingCurationhttps://w3id.org/health-ri/semantic-interoperabilityHealth-RI Semantic Interoperability Initiativehttps://creativecommons.org/licenses/by/4.0/</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" t="str">
         <f>"hrim:"&amp;Table4[[#This Row],[CRC-32]]</f>
         <v>hrim:</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="Z4" t="str">
-        <f>_xlfn.CONCAT(Table3[[#This Row],[mapping_date]])</f>
-        <v/>
-      </c>
-      <c r="AA4" s="6"/>
-      <c r="AB4" t="str">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="str">
+        <f>_xlfn.CONCAT(Table1[[#This Row],[subject_id]],Table1[[#This Row],[predicate_id]],Table1[[#This Row],[object_id]],Table1[[#This Row],[mapping_justification]],Table1[[#This Row],[author_id]],Table1[[#This Row],[reviewer_id]],Table1[[#This Row],[creator_id]],Table1[[#This Row],[creator_label]],Table1[[#This Row],[license]],Table1[[#This Row],[object_source_version]],Table1[[#This Row],[mapping_date]])</f>
+        <v>semapv:ManualMappingCurationhttps://w3id.org/health-ri/semantic-interoperabilityHealth-RI Semantic Interoperability Initiativehttps://creativecommons.org/licenses/by/4.0/</v>
+      </c>
+      <c r="B4" s="6"/>
+      <c r="C4" t="str">
         <f>"hrim:"&amp;Table4[[#This Row],[CRC-32]]</f>
         <v>hrim:</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A1:C1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <tableParts count="2">
+  <tableParts count="1">
     <tablePart r:id="rId2"/>
-    <tablePart r:id="rId3"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE6291F3-744E-4F97-AF6C-F3AD3689AF5B}">
+  <sheetPr>
+    <tabColor theme="7" tint="0.79998168889431442"/>
+  </sheetPr>
+  <dimension ref="B2:C12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="19" customWidth="1"/>
+    <col min="3" max="3" width="57.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="C2" s="20"/>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B3" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B4" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="C4" s="17">
+        <v>46108</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="C7" s="13"/>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B8" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B9" s="9"/>
+      <c r="C9" s="8" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B10" s="10"/>
+      <c r="C10" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B11" s="10"/>
+      <c r="C11" s="8" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B12" s="11"/>
+      <c r="C12" s="8" t="s">
+        <v>79</v>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
+  <mergeCells count="2">
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>